<commit_message>
Excel de pruebas: DEF-10 cerrado y ciclo 3 de verificación
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pruebas/PC09-PC10_Gestion_Pruebas_HU-004.xlsx
+++ b/pruebas/PC09-PC10_Gestion_Pruebas_HU-004.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1267" uniqueCount="507">
   <si>
     <t>Gestión de pruebas – HU-004 Registro de mermas justificadas</t>
   </si>
@@ -89,7 +89,7 @@
     <t>Ciclo</t>
   </si>
   <si>
-    <t>Ciclo 1 = primera ejecución · Ciclo 2 = re-ejecución tras corregir los defectos (regresión).</t>
+    <t>Ciclo 1 = primera ejecución · Ciclo 2 = re-ejecución tras corregir los defectos (regresión) · Ciclo 3 = verificación de DEF-10 tras habilitar TCP/IP (25/10/2026).</t>
   </si>
   <si>
     <t>Criterios de aceptación</t>
@@ -143,7 +143,7 @@
     <t>Generado</t>
   </si>
   <si>
-    <t>Desde las evidencias en pruebas/evidencias/ el 2026-10-24 00:12 (hora de Lima).</t>
+    <t>Desde las evidencias en pruebas/evidencias/ el 2026-10-24 19:33 (hora de Lima).</t>
   </si>
   <si>
     <t>PC 9 – Casos de prueba de la HU-004 (y regresión de modelos)</t>
@@ -860,6 +860,42 @@
     <t>EJ-022</t>
   </si>
   <si>
+    <t>2026-10-24 19:32</t>
+  </si>
+  <si>
+    <t>AJU-2026-00005 registrado; stock 96 → 94; historial 4 → 5 filas Verificación de DEF-10: puerto 1433 y pool de 10 conexiones.</t>
+  </si>
+  <si>
+    <t>DEF-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pruebas/evidencias/pc08/2026-10-25T00-32-11/01-login.png
+pruebas/evidencias/pc08/2026-10-25T00-32-11/02-modulo-ajustes.png
+pruebas/evidencias/pc08/2026-10-25T00-32-11/03-formulario-merma.png
+pruebas/evidencias/pc08/2026-10-25T00-32-11/04-merma-registrada.png</t>
+  </si>
+  <si>
+    <t>EJ-023</t>
+  </si>
+  <si>
+    <t>Mensaje mostrado: "La justificación técnica debe tener al menos 10 caracteres." Verificación de DEF-10: puerto 1433 y pool de 10 conexiones.</t>
+  </si>
+  <si>
+    <t>pruebas/evidencias/pc08/2026-10-25T00-32-11/05-error-justificacion-corta.png</t>
+  </si>
+  <si>
+    <t>EJ-024</t>
+  </si>
+  <si>
+    <t>Stock 1, solicitado 2: "No se puede descontar más del stock actual (1 unid.)." Verificación de DEF-10: puerto 1433 y pool de 10 conexiones.</t>
+  </si>
+  <si>
+    <t>pruebas/evidencias/pc08/2026-10-25T00-32-11/06-error-stock-insuficiente.png</t>
+  </si>
+  <si>
+    <t>EJ-025</t>
+  </si>
+  <si>
     <t>2026-10-24 00:06</t>
   </si>
   <si>
@@ -872,7 +908,7 @@
     <t>pruebas/evidencias/pc10/api-2026-10-24T05-06-39.json</t>
   </si>
   <si>
-    <t>EJ-023</t>
+    <t>EJ-026</t>
   </si>
   <si>
     <t>201; folios AJU-2026-00002 y AJU-2026-00003</t>
@@ -881,67 +917,67 @@
     <t>DEF-01</t>
   </si>
   <si>
-    <t>EJ-024</t>
+    <t>EJ-027</t>
   </si>
   <si>
     <t>400; La justificación técnica es obligatoria.</t>
   </si>
   <si>
-    <t>EJ-025</t>
+    <t>EJ-028</t>
   </si>
   <si>
     <t>400; La justificación técnica debe tener al menos 10 caracteres.</t>
   </si>
   <si>
-    <t>EJ-026</t>
+    <t>EJ-029</t>
   </si>
   <si>
     <t>400; La cantidad del ajuste debe ser un número entero mayor a 0.</t>
   </si>
   <si>
-    <t>EJ-027</t>
+    <t>EJ-030</t>
   </si>
   <si>
     <t>400; No se puede descontar más del stock actual (1 unid.).</t>
   </si>
   <si>
-    <t>EJ-028</t>
+    <t>EJ-031</t>
   </si>
   <si>
     <t>400; El producto especificado no existe o está inactivo.</t>
   </si>
   <si>
-    <t>EJ-029</t>
+    <t>EJ-032</t>
   </si>
   <si>
     <t>403; No tiene permisos para esta acción.</t>
   </si>
   <si>
-    <t>EJ-030</t>
+    <t>EJ-033</t>
   </si>
   <si>
     <t>401; Sesión no iniciada.</t>
   </si>
   <si>
-    <t>EJ-031</t>
+    <t>EJ-034</t>
   </si>
   <si>
     <t>201; stock 91 → 96</t>
   </si>
   <si>
-    <t>EJ-032</t>
+    <t>EJ-035</t>
   </si>
   <si>
     <t>200; 4 ajustes; incluye AJU-2026-00002, AJU-2026-00003, AJU-2026-00004: true</t>
   </si>
   <si>
-    <t>EJ-033</t>
+    <t>EJ-036</t>
   </si>
   <si>
     <t>3 asientos: AJU-2026-00002, AJU-2026-00003, AJU-2026-00004</t>
   </si>
   <si>
-    <t>EJ-034</t>
+    <t>EJ-037</t>
   </si>
   <si>
     <t>0 registros; ej.: MOVIMIENTO_MERMA por Jorge Luis Paredes Soto el 2026-10-24T05:06:08.750Z — Producto: Tablero Melamina Vesto Roble Cendra 18mm (SKU: 1), Cantidad: 2, Stock Anterior: 95, Stock Nuevo: 93, Doc: AJU-2026-00002</t>
@@ -950,21 +986,12 @@
     <t>DEF-09</t>
   </si>
   <si>
-    <t>EJ-035</t>
+    <t>EJ-038</t>
   </si>
   <si>
     <t>pruebas/evidencias/pc10/api-2026-10-24T05-08-27.json</t>
   </si>
   <si>
-    <t>EJ-036</t>
-  </si>
-  <si>
-    <t>EJ-037</t>
-  </si>
-  <si>
-    <t>EJ-038</t>
-  </si>
-  <si>
     <t>EJ-039</t>
   </si>
   <si>
@@ -992,9 +1019,63 @@
     <t>EJ-047</t>
   </si>
   <si>
+    <t>EJ-048</t>
+  </si>
+  <si>
+    <t>EJ-049</t>
+  </si>
+  <si>
+    <t>EJ-050</t>
+  </si>
+  <si>
     <t>3 registros; ej.: MOVIMIENTO_MERMA por Jorge Luis Paredes Soto el 2026-10-24T05:07:51.781Z — Producto: Tablero Melamina Vesto Roble Cendra 18mm (SKU: MEL-VES-ROB-18), Cantidad: 2, Stock Anterior: 95, Stock Nuevo: 93, Doc: AJU-2026-00002 | [Ajuste] Tablero desportillado: Golpe de montacargas en la esquina durante la descarga</t>
   </si>
   <si>
+    <t>EJ-051</t>
+  </si>
+  <si>
+    <t>pruebas/evidencias/pc10/api-2026-10-25T00-32-07.json</t>
+  </si>
+  <si>
+    <t>EJ-052</t>
+  </si>
+  <si>
+    <t>EJ-053</t>
+  </si>
+  <si>
+    <t>EJ-054</t>
+  </si>
+  <si>
+    <t>EJ-055</t>
+  </si>
+  <si>
+    <t>EJ-056</t>
+  </si>
+  <si>
+    <t>EJ-057</t>
+  </si>
+  <si>
+    <t>EJ-058</t>
+  </si>
+  <si>
+    <t>EJ-059</t>
+  </si>
+  <si>
+    <t>EJ-060</t>
+  </si>
+  <si>
+    <t>EJ-061</t>
+  </si>
+  <si>
+    <t>EJ-062</t>
+  </si>
+  <si>
+    <t>EJ-063</t>
+  </si>
+  <si>
+    <t>3 registros; ej.: MOVIMIENTO_MERMA por Jorge Luis Paredes Soto el 2026-10-25T00:32:06.780Z — Producto: Tablero Melamina Vesto Roble Cendra 18mm (SKU: MEL-VES-ROB-18), Cantidad: 2, Stock Anterior: 95, Stock Nuevo: 93, Doc: AJU-2026-00002 | [Ajuste] Tablero desportillado: Golpe de montacargas en la esquina durante la descarga</t>
+  </si>
+  <si>
     <t>PC 10 – Registro de defectos</t>
   </si>
   <si>
@@ -1229,9 +1310,6 @@
     <t>Descripción con CodigoSKU y observación (commit b4e05f0)</t>
   </si>
   <si>
-    <t>DEF-10</t>
-  </si>
-  <si>
     <t>Ambiente local: SQL Server sin TCP/IP, solo acepta 1 conexión</t>
   </si>
   <si>
@@ -1250,13 +1328,13 @@
     <t>Verificación manual de la PC 6</t>
   </si>
   <si>
-    <t>— (ambiente)</t>
-  </si>
-  <si>
-    <t>Paliativo: DB_POOL_MAX=1. Pendiente: habilitar TCP/IP (1433) y usar un usuario sin sysadmin.</t>
-  </si>
-  <si>
-    <t>Abierto</t>
+    <t>CP-HU4-01 a CP-HU4-16 (ciclo 3)</t>
+  </si>
+  <si>
+    <t>TCP/IP habilitado en MSSQLSERVER (puerto 1433); configuración y plantillas con DB_PORT=1433 y sin DB_POOL_MAX (commit ac88fe7). Recomendado además: usuario de BD local sin rol sysadmin.</t>
+  </si>
+  <si>
+    <t>2026-10-25</t>
   </si>
   <si>
     <t>DEF-11</t>
@@ -1400,6 +1478,9 @@
     <t>Ciclo 2</t>
   </si>
   <si>
+    <t>Ciclo 3</t>
+  </si>
+  <si>
     <t>Ejecuciones</t>
   </si>
   <si>
@@ -1415,7 +1496,7 @@
     <t>% de aprobación</t>
   </si>
   <si>
-    <t>Ciclo 2 = re-ejecución tras corregir los defectos</t>
+    <t>Ciclo 2 = regresión tras corregir defectos · Ciclo 3 = verificación de DEF-10</t>
   </si>
   <si>
     <t>Defectos (PC 10)</t>
@@ -3140,7 +3221,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -3940,16 +4021,16 @@
         <v>277</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="C25" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>278</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>279</v>
+        <v>251</v>
       </c>
       <c r="F25" s="11" t="s">
         <v>219</v>
@@ -3958,13 +4039,13 @@
         <v>220</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>222</v>
       </c>
       <c r="J25" s="10" t="s">
-        <v>12</v>
+        <v>280</v>
       </c>
       <c r="K25" s="10" t="s">
         <v>281</v>
@@ -3975,16 +4056,16 @@
         <v>282</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="C26" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D26" s="9" t="s">
         <v>278</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>279</v>
+        <v>251</v>
       </c>
       <c r="F26" s="11" t="s">
         <v>219</v>
@@ -3999,10 +4080,10 @@
         <v>222</v>
       </c>
       <c r="J26" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K26" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="K26" s="9" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -4010,16 +4091,16 @@
         <v>285</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="C27" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>278</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>279</v>
+        <v>251</v>
       </c>
       <c r="F27" s="11" t="s">
         <v>219</v>
@@ -4034,27 +4115,27 @@
         <v>222</v>
       </c>
       <c r="J27" s="10" t="s">
-        <v>12</v>
+        <v>280</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="C28" s="9">
         <v>1</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F28" s="11" t="s">
         <v>219</v>
@@ -4063,7 +4144,7 @@
         <v>220</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="I28" s="9" t="s">
         <v>222</v>
@@ -4072,24 +4153,24 @@
         <v>12</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="C29" s="10">
         <v>1</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F29" s="11" t="s">
         <v>219</v>
@@ -4098,33 +4179,33 @@
         <v>220</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="I29" s="10" t="s">
         <v>222</v>
       </c>
       <c r="J29" s="10" t="s">
-        <v>12</v>
+        <v>295</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C30" s="9">
         <v>1</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F30" s="11" t="s">
         <v>219</v>
@@ -4133,7 +4214,7 @@
         <v>220</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="I30" s="9" t="s">
         <v>222</v>
@@ -4142,24 +4223,24 @@
         <v>12</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="C31" s="10">
         <v>1</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F31" s="11" t="s">
         <v>219</v>
@@ -4168,7 +4249,7 @@
         <v>220</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="I31" s="10" t="s">
         <v>222</v>
@@ -4177,24 +4258,24 @@
         <v>12</v>
       </c>
       <c r="K31" s="10" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C32" s="9">
         <v>1</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F32" s="11" t="s">
         <v>219</v>
@@ -4203,7 +4284,7 @@
         <v>220</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="I32" s="9" t="s">
         <v>222</v>
@@ -4212,24 +4293,24 @@
         <v>12</v>
       </c>
       <c r="K32" s="9" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="10" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="C33" s="10">
         <v>1</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F33" s="11" t="s">
         <v>219</v>
@@ -4238,7 +4319,7 @@
         <v>220</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="I33" s="10" t="s">
         <v>222</v>
@@ -4247,24 +4328,24 @@
         <v>12</v>
       </c>
       <c r="K33" s="10" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="C34" s="9">
         <v>1</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F34" s="11" t="s">
         <v>219</v>
@@ -4273,7 +4354,7 @@
         <v>220</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="I34" s="9" t="s">
         <v>222</v>
@@ -4282,24 +4363,24 @@
         <v>12</v>
       </c>
       <c r="K34" s="9" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="10" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="C35" s="10">
         <v>1</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F35" s="11" t="s">
         <v>219</v>
@@ -4308,7 +4389,7 @@
         <v>220</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="I35" s="10" t="s">
         <v>222</v>
@@ -4317,24 +4398,24 @@
         <v>12</v>
       </c>
       <c r="K35" s="10" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="C36" s="9">
         <v>1</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E36" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F36" s="11" t="s">
         <v>219</v>
@@ -4343,7 +4424,7 @@
         <v>220</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="I36" s="9" t="s">
         <v>222</v>
@@ -4352,24 +4433,24 @@
         <v>12</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="C37" s="10">
         <v>1</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F37" s="11" t="s">
         <v>219</v>
@@ -4378,33 +4459,33 @@
         <v>220</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="I37" s="10" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="J37" s="10" t="s">
-        <v>307</v>
+        <v>12</v>
       </c>
       <c r="K37" s="10" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>82</v>
+        <v>143</v>
       </c>
       <c r="C38" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F38" s="11" t="s">
         <v>219</v>
@@ -4413,7 +4494,7 @@
         <v>220</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>280</v>
+        <v>313</v>
       </c>
       <c r="I38" s="9" t="s">
         <v>222</v>
@@ -4422,24 +4503,24 @@
         <v>12</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>309</v>
+        <v>292</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>92</v>
+        <v>151</v>
       </c>
       <c r="C39" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F39" s="11" t="s">
         <v>219</v>
@@ -4448,33 +4529,33 @@
         <v>220</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>283</v>
+        <v>315</v>
       </c>
       <c r="I39" s="10" t="s">
         <v>222</v>
       </c>
       <c r="J39" s="10" t="s">
-        <v>284</v>
+        <v>12</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>309</v>
+        <v>292</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>100</v>
+        <v>158</v>
       </c>
       <c r="C40" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F40" s="11" t="s">
         <v>219</v>
@@ -4483,24 +4564,24 @@
         <v>220</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>286</v>
+        <v>317</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>12</v>
+        <v>318</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>309</v>
+        <v>292</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>106</v>
+        <v>82</v>
       </c>
       <c r="C41" s="10">
         <v>2</v>
@@ -4509,7 +4590,7 @@
         <v>270</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F41" s="11" t="s">
         <v>219</v>
@@ -4518,7 +4599,7 @@
         <v>220</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="I41" s="10" t="s">
         <v>222</v>
@@ -4527,15 +4608,15 @@
         <v>12</v>
       </c>
       <c r="K41" s="10" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="C42" s="9">
         <v>2</v>
@@ -4544,7 +4625,7 @@
         <v>270</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F42" s="11" t="s">
         <v>219</v>
@@ -4553,24 +4634,24 @@
         <v>220</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="I42" s="9" t="s">
         <v>222</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>12</v>
+        <v>295</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="C43" s="10">
         <v>2</v>
@@ -4579,7 +4660,7 @@
         <v>270</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F43" s="11" t="s">
         <v>219</v>
@@ -4588,7 +4669,7 @@
         <v>220</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="I43" s="10" t="s">
         <v>222</v>
@@ -4597,15 +4678,15 @@
         <v>12</v>
       </c>
       <c r="K43" s="10" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="C44" s="9">
         <v>2</v>
@@ -4614,7 +4695,7 @@
         <v>270</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F44" s="11" t="s">
         <v>219</v>
@@ -4623,7 +4704,7 @@
         <v>220</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="I44" s="9" t="s">
         <v>222</v>
@@ -4632,15 +4713,15 @@
         <v>12</v>
       </c>
       <c r="K44" s="9" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C45" s="10">
         <v>2</v>
@@ -4649,7 +4730,7 @@
         <v>270</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F45" s="11" t="s">
         <v>219</v>
@@ -4658,7 +4739,7 @@
         <v>220</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="I45" s="10" t="s">
         <v>222</v>
@@ -4667,15 +4748,15 @@
         <v>12</v>
       </c>
       <c r="K45" s="10" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="C46" s="9">
         <v>2</v>
@@ -4684,7 +4765,7 @@
         <v>270</v>
       </c>
       <c r="E46" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F46" s="11" t="s">
         <v>219</v>
@@ -4693,7 +4774,7 @@
         <v>220</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="I46" s="9" t="s">
         <v>222</v>
@@ -4702,15 +4783,15 @@
         <v>12</v>
       </c>
       <c r="K46" s="9" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="C47" s="10">
         <v>2</v>
@@ -4719,7 +4800,7 @@
         <v>270</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F47" s="11" t="s">
         <v>219</v>
@@ -4728,7 +4809,7 @@
         <v>220</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="I47" s="10" t="s">
         <v>222</v>
@@ -4737,15 +4818,15 @@
         <v>12</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="C48" s="9">
         <v>2</v>
@@ -4754,7 +4835,7 @@
         <v>270</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F48" s="11" t="s">
         <v>219</v>
@@ -4763,7 +4844,7 @@
         <v>220</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="I48" s="9" t="s">
         <v>222</v>
@@ -4772,15 +4853,15 @@
         <v>12</v>
       </c>
       <c r="K48" s="9" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
       <c r="C49" s="10">
         <v>2</v>
@@ -4789,7 +4870,7 @@
         <v>270</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F49" s="11" t="s">
         <v>219</v>
@@ -4798,7 +4879,7 @@
         <v>220</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="I49" s="10" t="s">
         <v>222</v>
@@ -4807,15 +4888,15 @@
         <v>12</v>
       </c>
       <c r="K49" s="10" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="C50" s="9">
         <v>2</v>
@@ -4824,7 +4905,7 @@
         <v>270</v>
       </c>
       <c r="E50" s="9" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="F50" s="11" t="s">
         <v>219</v>
@@ -4833,21 +4914,581 @@
         <v>220</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="I50" s="9" t="s">
         <v>222</v>
       </c>
       <c r="J50" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="K50" s="9" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C51" s="10">
+        <v>2</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G51" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="I51" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J51" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="K51" s="10" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C52" s="9">
+        <v>2</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F52" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H52" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="I52" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J52" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="K52" s="9" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="C53" s="10">
+        <v>2</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="E53" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F53" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G53" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J53" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="K53" s="10" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="9" t="s">
+        <v>334</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C54" s="9">
+        <v>3</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F54" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H54" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="I54" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J54" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K54" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C55" s="10">
+        <v>3</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F55" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G55" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H55" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="I55" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J55" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="K55" s="10" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" s="9">
+        <v>3</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F56" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="I56" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J56" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K56" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="B57" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" s="10">
+        <v>3</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F57" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G57" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H57" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J57" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="K57" s="10" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C58" s="9">
+        <v>3</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F58" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="I58" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J58" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K58" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="10" t="s">
+        <v>340</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="C59" s="10">
+        <v>3</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F59" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G59" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H59" s="10" t="s">
+        <v>303</v>
+      </c>
+      <c r="I59" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J59" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="K59" s="10" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C60" s="9">
+        <v>3</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F60" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="I60" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J60" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K60" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="B61" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="C61" s="10">
+        <v>3</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E61" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G61" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H61" s="10" t="s">
         <v>307</v>
       </c>
-      <c r="K50" s="9" t="s">
+      <c r="I61" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J61" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="K61" s="10" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C62" s="9">
+        <v>3</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F62" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G62" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H62" s="9" t="s">
         <v>309</v>
       </c>
+      <c r="I62" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J62" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K62" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="B63" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C63" s="10">
+        <v>3</v>
+      </c>
+      <c r="D63" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E63" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G63" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H63" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="I63" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J63" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="K63" s="10" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="C64" s="9">
+        <v>3</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F64" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H64" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="I64" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J64" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K64" s="9" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="B65" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="C65" s="10">
+        <v>3</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E65" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="F65" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G65" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="H65" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="I65" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J65" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="K65" s="10" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" s="9" t="s">
+        <v>347</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C66" s="9">
+        <v>3</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E66" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="F66" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="G66" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="H66" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="I66" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="J66" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="K66" s="9" t="s">
+        <v>335</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:K50"/>
-  <conditionalFormatting sqref="I4:I50">
+  <autoFilter ref="A3:K66"/>
+  <conditionalFormatting sqref="I4:I66">
     <cfRule type="containsText" dxfId="0" priority="1">
       <formula>NOT(ISERROR(SEARCH("Aprobado",I4)))</formula>
     </cfRule>
@@ -4865,10 +5506,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Use: Aprobado, Fallido, Bloqueado" sqref="I10:I50">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Use: Aprobado, Fallido, Bloqueado" sqref="I10:I66">
       <formula1>"Aprobado,Fallido,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Use: Aprobado, Fallido, Bloqueado" sqref="I4:I50">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Use: Aprobado, Fallido, Bloqueado" sqref="I4:I66">
       <formula1>"Aprobado,Fallido,Bloqueado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4899,12 +5540,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>323</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>324</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -4915,10 +5556,10 @@
         <v>47</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>325</v>
+        <v>351</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>326</v>
+        <v>352</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>54</v>
@@ -4927,25 +5568,25 @@
         <v>212</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>327</v>
+        <v>353</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>15</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="J3" s="8" t="s">
-        <v>329</v>
+        <v>355</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>330</v>
+        <v>356</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>331</v>
+        <v>357</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>332</v>
+        <v>358</v>
       </c>
       <c r="N3" s="8" t="s">
         <v>210</v>
@@ -4956,22 +5597,22 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>333</v>
+        <v>359</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>334</v>
+        <v>360</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>335</v>
+        <v>361</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>336</v>
+        <v>362</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>337</v>
+        <v>363</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>96</v>
@@ -4980,45 +5621,45 @@
         <v>61</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>338</v>
+        <v>364</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>92</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>340</v>
+        <v>366</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="N4" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>343</v>
+        <v>369</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>344</v>
+        <v>370</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>345</v>
+        <v>371</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>347</v>
+        <v>373</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>348</v>
+        <v>374</v>
       </c>
       <c r="G5" s="10" t="s">
         <v>61</v>
@@ -5027,45 +5668,45 @@
         <v>61</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>349</v>
+        <v>375</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>350</v>
+        <v>376</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>351</v>
+        <v>377</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>352</v>
+        <v>378</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>353</v>
+        <v>379</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>354</v>
+        <v>380</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>355</v>
+        <v>381</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>356</v>
+        <v>382</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>357</v>
+        <v>383</v>
       </c>
       <c r="G6" s="9" t="s">
         <v>96</v>
@@ -5074,25 +5715,25 @@
         <v>61</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>349</v>
+        <v>375</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>358</v>
+        <v>384</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>359</v>
+        <v>385</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O6" s="9" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -5100,19 +5741,19 @@
         <v>232</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>360</v>
+        <v>386</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>361</v>
+        <v>387</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>362</v>
+        <v>388</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>363</v>
+        <v>389</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>364</v>
+        <v>390</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>96</v>
@@ -5121,45 +5762,45 @@
         <v>96</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>365</v>
+        <v>391</v>
       </c>
       <c r="J7" s="10" t="s">
         <v>187</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>366</v>
+        <v>392</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O7" s="10" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>367</v>
+        <v>393</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>368</v>
+        <v>394</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>369</v>
+        <v>395</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>370</v>
+        <v>396</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>363</v>
+        <v>389</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>364</v>
+        <v>390</v>
       </c>
       <c r="G8" s="9" t="s">
         <v>96</v>
@@ -5168,45 +5809,45 @@
         <v>96</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>371</v>
+        <v>397</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>182</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>372</v>
+        <v>398</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O8" s="9" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>373</v>
+        <v>399</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>374</v>
+        <v>400</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>375</v>
+        <v>401</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>376</v>
+        <v>402</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>363</v>
+        <v>389</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>377</v>
+        <v>403</v>
       </c>
       <c r="G9" s="10" t="s">
         <v>96</v>
@@ -5215,25 +5856,25 @@
         <v>96</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>371</v>
+        <v>397</v>
       </c>
       <c r="J9" s="10" t="s">
         <v>182</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L9" s="10" t="s">
-        <v>378</v>
+        <v>404</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O9" s="10" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -5241,19 +5882,19 @@
         <v>235</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>379</v>
+        <v>405</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>380</v>
+        <v>406</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>381</v>
+        <v>407</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>382</v>
+        <v>408</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>383</v>
+        <v>409</v>
       </c>
       <c r="G10" s="9" t="s">
         <v>195</v>
@@ -5262,25 +5903,25 @@
         <v>195</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>384</v>
+        <v>410</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>192</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>385</v>
+        <v>411</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="N10" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O10" s="9" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
@@ -5288,19 +5929,19 @@
         <v>253</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>386</v>
+        <v>412</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>387</v>
+        <v>413</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>388</v>
+        <v>414</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>389</v>
+        <v>415</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>390</v>
+        <v>416</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>96</v>
@@ -5309,45 +5950,45 @@
         <v>96</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>391</v>
+        <v>417</v>
       </c>
       <c r="J11" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>392</v>
+        <v>418</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>393</v>
+        <v>419</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>392</v>
+        <v>418</v>
       </c>
       <c r="N11" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O11" s="10" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>394</v>
+        <v>420</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>395</v>
+        <v>421</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>396</v>
+        <v>422</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>397</v>
+        <v>423</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>398</v>
+        <v>424</v>
       </c>
       <c r="G12" s="9" t="s">
         <v>96</v>
@@ -5356,45 +5997,45 @@
         <v>61</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>399</v>
+        <v>425</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>158</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>392</v>
+        <v>418</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>400</v>
+        <v>426</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>392</v>
+        <v>418</v>
       </c>
       <c r="N12" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O12" s="9" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>401</v>
+        <v>280</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>402</v>
+        <v>427</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>403</v>
+        <v>428</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>404</v>
+        <v>429</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>405</v>
+        <v>430</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>406</v>
+        <v>431</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>61</v>
@@ -5403,45 +6044,45 @@
         <v>61</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>407</v>
+        <v>432</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>408</v>
+        <v>433</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>409</v>
+        <v>434</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>12</v>
+        <v>435</v>
       </c>
       <c r="N13" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O13" s="10" t="s">
-        <v>410</v>
+        <v>368</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>411</v>
+        <v>436</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>412</v>
+        <v>437</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>413</v>
+        <v>438</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>414</v>
+        <v>439</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>415</v>
+        <v>440</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>416</v>
+        <v>441</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>61</v>
@@ -5450,45 +6091,45 @@
         <v>96</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>417</v>
+        <v>442</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>418</v>
+        <v>443</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>419</v>
+        <v>444</v>
       </c>
       <c r="M14" s="9" t="s">
         <v>12</v>
       </c>
       <c r="N14" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O14" s="9" t="s">
-        <v>420</v>
+        <v>445</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>421</v>
+        <v>446</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>422</v>
+        <v>447</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>423</v>
+        <v>448</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>424</v>
+        <v>449</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>425</v>
+        <v>450</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>426</v>
+        <v>451</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>96</v>
@@ -5497,45 +6138,45 @@
         <v>96</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>418</v>
+        <v>443</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>419</v>
+        <v>444</v>
       </c>
       <c r="M15" s="10" t="s">
         <v>12</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>420</v>
+        <v>445</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>428</v>
+        <v>453</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>429</v>
+        <v>454</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>430</v>
+        <v>455</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>431</v>
+        <v>456</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>432</v>
+        <v>457</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>433</v>
+        <v>458</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>96</v>
@@ -5544,45 +6185,45 @@
         <v>96</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>434</v>
+        <v>459</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>435</v>
+        <v>460</v>
       </c>
       <c r="M16" s="9" t="s">
         <v>12</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O16" s="9" t="s">
-        <v>420</v>
+        <v>445</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>436</v>
+        <v>461</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>437</v>
+        <v>462</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>438</v>
+        <v>463</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>439</v>
+        <v>464</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>440</v>
+        <v>465</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>441</v>
+        <v>466</v>
       </c>
       <c r="G17" s="10" t="s">
         <v>61</v>
@@ -5591,25 +6232,25 @@
         <v>61</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>427</v>
+        <v>452</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>442</v>
+        <v>467</v>
       </c>
       <c r="K17" s="10" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>443</v>
+        <v>468</v>
       </c>
       <c r="M17" s="10" t="s">
         <v>12</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>420</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>
@@ -5652,30 +6293,30 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
-    <col min="2" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="2" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>444</v>
+        <v>469</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>446</v>
+        <v>471</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>447</v>
+        <v>472</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>12</v>
@@ -5686,188 +6327,210 @@
       <c r="E4" s="12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>448</v>
+        <v>473</v>
       </c>
       <c r="B5" s="14">
         <f>COUNTA('Casos de Prueba'!$A$4:$A$25)</f>
         <v>22</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>449</v>
+        <v>474</v>
       </c>
       <c r="B6" s="14">
         <f>COUNTIF('Casos de Prueba'!$F$4:$F$25,"Alta")</f>
         <v>12</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>450</v>
+        <v>475</v>
       </c>
       <c r="B7" s="14">
         <f>COUNTIF('Casos de Prueba'!$F$4:$F$25,"Media")</f>
         <v>9</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>451</v>
+        <v>476</v>
       </c>
       <c r="B8" s="14">
         <f>COUNTIF('Casos de Prueba'!$F$4:$F$25,"Baja")</f>
         <v>1</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>452</v>
+        <v>477</v>
       </c>
       <c r="B9" s="14">
         <f>COUNTIF('Casos de Prueba'!$D$4:$D$25,"Funcional E2E")</f>
         <v>3</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>453</v>
+        <v>478</v>
       </c>
       <c r="B10" s="14">
         <f>COUNTIF('Casos de Prueba'!$D$4:$D$25,"API")</f>
         <v>13</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>454</v>
+        <v>479</v>
       </c>
       <c r="B11" s="14">
         <f>COUNTIF('Casos de Prueba'!$D$4:$D$25,"Unitaria")</f>
         <v>6</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>455</v>
+        <v>480</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>456</v>
+        <v>481</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>457</v>
+        <v>482</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>483</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>458</v>
+        <v>484</v>
       </c>
       <c r="B14" s="14">
-        <f>COUNTIF('Ejecución'!$C$4:$C$50,1)</f>
+        <f>COUNTIF('Ejecución'!$C$4:$C$66,1)</f>
         <v>22</v>
       </c>
       <c r="C14" s="14">
-        <f>COUNTIF('Ejecución'!$C$4:$C$50,2)</f>
+        <f>COUNTIF('Ejecución'!$C$4:$C$66,2)</f>
         <v>25</v>
       </c>
       <c r="D14" s="14">
-        <f>COUNTA('Ejecución'!$A$4:$A$50)</f>
-        <v>47</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <f>COUNTIF('Ejecución'!$C$4:$C$66,3)</f>
+        <v>16</v>
+      </c>
+      <c r="E14" s="14">
+        <f>COUNTA('Ejecución'!$A$4:$A$66)</f>
+        <v>63</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>459</v>
+        <v>485</v>
       </c>
       <c r="B15" s="14">
-        <f>COUNTIFS('Ejecución'!$C$4:$C$50,1,'Ejecución'!$I$4:$I$50,"Aprobado")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,1,'Ejecución'!$I$4:$I$66,"Aprobado")</f>
         <v>18</v>
       </c>
       <c r="C15" s="14">
-        <f>COUNTIFS('Ejecución'!$C$4:$C$50,2,'Ejecución'!$I$4:$I$50,"Aprobado")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,2,'Ejecución'!$I$4:$I$66,"Aprobado")</f>
         <v>25</v>
       </c>
       <c r="D15" s="14">
-        <f>COUNTIF('Ejecución'!$I$4:$I$50,"Aprobado")</f>
-        <v>43</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,3,'Ejecución'!$I$4:$I$66,"Aprobado")</f>
+        <v>16</v>
+      </c>
+      <c r="E15" s="14">
+        <f>COUNTIF('Ejecución'!$I$4:$I$66,"Aprobado")</f>
+        <v>59</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>460</v>
+        <v>486</v>
       </c>
       <c r="B16" s="14">
-        <f>COUNTIFS('Ejecución'!$C$4:$C$50,1,'Ejecución'!$I$4:$I$50,"Fallido")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,1,'Ejecución'!$I$4:$I$66,"Fallido")</f>
         <v>4</v>
       </c>
       <c r="C16" s="14">
-        <f>COUNTIFS('Ejecución'!$C$4:$C$50,2,'Ejecución'!$I$4:$I$50,"Fallido")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,2,'Ejecución'!$I$4:$I$66,"Fallido")</f>
         <v>0</v>
       </c>
       <c r="D16" s="14">
-        <f>COUNTIF('Ejecución'!$I$4:$I$50,"Fallido")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,3,'Ejecución'!$I$4:$I$66,"Fallido")</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="14">
+        <f>COUNTIF('Ejecución'!$I$4:$I$66,"Fallido")</f>
         <v>4</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>461</v>
+        <v>487</v>
       </c>
       <c r="B17" s="14">
-        <f>COUNTIFS('Ejecución'!$C$4:$C$50,1,'Ejecución'!$I$4:$I$50,"Bloqueado")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,1,'Ejecución'!$I$4:$I$66,"Bloqueado")</f>
         <v>0</v>
       </c>
       <c r="C17" s="14">
-        <f>COUNTIFS('Ejecución'!$C$4:$C$50,2,'Ejecución'!$I$4:$I$50,"Bloqueado")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,2,'Ejecución'!$I$4:$I$66,"Bloqueado")</f>
         <v>0</v>
       </c>
       <c r="D17" s="14">
-        <f>COUNTIF('Ejecución'!$I$4:$I$50,"Bloqueado")</f>
+        <f>COUNTIFS('Ejecución'!$C$4:$C$66,3,'Ejecución'!$I$4:$I$66,"Bloqueado")</f>
         <v>0</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="14">
+        <f>COUNTIF('Ejecución'!$I$4:$I$66,"Bloqueado")</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>462</v>
+        <v>488</v>
       </c>
       <c r="B18" s="15">
         <f>IFERROR(B15/B14,0)</f>
@@ -5879,18 +6542,22 @@
       </c>
       <c r="D18" s="15">
         <f>IFERROR(D15/D14,0)</f>
-        <v>0.9148936170212766</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="E18" s="15">
+        <f>IFERROR(E15/E14,0)</f>
+        <v>0.9365079365079365</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>464</v>
+        <v>490</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>447</v>
+        <v>472</v>
       </c>
       <c r="C20" s="12" t="s">
         <v>12</v>
@@ -5901,111 +6568,117 @@
       <c r="E20" s="12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>465</v>
+        <v>491</v>
       </c>
       <c r="B21" s="14">
         <f>COUNTA('Defectos'!$A$4:$A$17)</f>
         <v>14</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="13" t="s">
-        <v>466</v>
+        <v>492</v>
       </c>
       <c r="B22" s="14">
         <f>COUNTIF('Defectos'!$G$4:$G$17,"Alta")</f>
         <v>4</v>
       </c>
-      <c r="E22" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>467</v>
+        <v>493</v>
       </c>
       <c r="B23" s="14">
         <f>COUNTIF('Defectos'!$G$4:$G$17,"Media")</f>
         <v>9</v>
       </c>
-      <c r="E23" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>468</v>
+        <v>494</v>
       </c>
       <c r="B24" s="14">
         <f>COUNTIF('Defectos'!$G$4:$G$17,"Baja")</f>
         <v>1</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>469</v>
+        <v>495</v>
       </c>
       <c r="B25" s="14">
         <f>COUNTIF('Defectos'!$O$4:$O$17,"Cerrado")</f>
-        <v>9</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>470</v>
+        <v>496</v>
       </c>
       <c r="B26" s="14">
         <f>COUNTIF('Defectos'!$O$4:$O$17,"Abierto")</f>
-        <v>1</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>471</v>
+        <v>497</v>
       </c>
       <c r="B27" s="14">
         <f>COUNTIF('Defectos'!$O$4:$O$17,"Diferido")</f>
         <v>4</v>
       </c>
-      <c r="E27" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>472</v>
+        <v>498</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>473</v>
+        <v>499</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>474</v>
+        <v>500</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>475</v>
+        <v>501</v>
       </c>
       <c r="E29" s="12" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>476</v>
+        <v>502</v>
       </c>
       <c r="B30" s="14">
         <v>93.38</v>
@@ -6017,13 +6690,13 @@
         <f>IF(B30&gt;=C30,"Sí","No")</f>
         <v>Sí</v>
       </c>
-      <c r="E30" s="2" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="2" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
-        <v>478</v>
+        <v>504</v>
       </c>
       <c r="B31" s="14">
         <v>96.29</v>
@@ -6035,13 +6708,13 @@
         <f>IF(B31&gt;=C31,"Sí","No")</f>
         <v>Sí</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" s="2" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
-        <v>479</v>
+        <v>505</v>
       </c>
       <c r="B32" s="14">
         <v>95.23</v>
@@ -6053,13 +6726,13 @@
         <f>IF(B32&gt;=C32,"Sí","No")</f>
         <v>Sí</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" s="2" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>480</v>
+        <v>506</v>
       </c>
       <c r="B33" s="14">
         <v>93.38</v>
@@ -6071,8 +6744,8 @@
         <f>IF(B33&gt;=C33,"Sí","No")</f>
         <v>Sí</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>477</v>
+      <c r="F33" s="2" t="s">
+        <v>503</v>
       </c>
     </row>
   </sheetData>

</xml_diff>